<commit_message>
Add owner-first tomato marginal cost column
</commit_message>
<xml_diff>
--- a/capabilities/marginal-analysis/model.xlsx
+++ b/capabilities/marginal-analysis/model.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/def2638157994097/Desktop/Economics/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{2C762524-61C6-445E-AC11-8DA69166658F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{B96F9A43-E369-43EC-BBE6-E2F35AF1AF09}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Inputs" sheetId="1" r:id="rId1"/>
@@ -105,7 +105,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="130">
   <si>
     <t>Decision Variables</t>
   </si>
@@ -404,6 +404,9 @@
     <t>Mesclun MC ($)</t>
   </si>
   <si>
+    <t>Tomato MC, owner-first ($)</t>
+  </si>
+  <si>
     <t>NOTE: this standalone schedule approximates marginal labor cost at the TEMP_RATE</t>
   </si>
   <si>
@@ -411,6 +414,15 @@
   </si>
   <si>
     <t>the Farm Profit Lab and note any material difference in your audit.</t>
+  </si>
+  <si>
+    <t>NOTE (added during audit): column I prices tomato labor the way spec Section 3 describes: the first OWNER_HRS at OWNER_RATE, any hours after that at TEMP_RATE. It is a tomatoes-grown-alone view.</t>
+  </si>
+  <si>
+    <t>Column C prices every hour at TEMP_RATE, so it never shows the owner-to-temp step-down. The material difference is tomato beds 1-5: owner-first MC peaks at bed 5 ($7,661), then falls at bed 6 ($4,906) once the 720 owner hours are used up.</t>
+  </si>
+  <si>
+    <t>From bed 6 on, columns C and I are identical. Carrot and mesclun are not repeated owner-first here: in the full farm the three crops share the 720 owner hours, so a crop-alone owner-first view would overstate their early-bed costs.</t>
   </si>
   <si>
     <t>Validation Rule</t>
@@ -1717,13 +1729,14 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G35"/>
+  <dimension ref="A1:I39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="7" width="17" customWidth="1"/>
+    <col min="9" max="9" width="26" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>90</v>
       </c>
@@ -1731,7 +1744,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>92</v>
       </c>
@@ -1753,8 +1766,11 @@
       <c r="G3" s="1" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I3" s="1" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>1</v>
       </c>
@@ -1782,8 +1798,12 @@
         <f>(F4*TEMP_RATE+MESCLUN_FERT)</f>
         <v>1671.015625</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I4">
+        <f>(MIN(B4,OWNER_HRS)*OWNER_RATE+MAX(0,B4-OWNER_HRS)*TEMP_RATE)+TOMATO_FERT</f>
+        <v>4317.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>2</v>
       </c>
@@ -1811,8 +1831,12 @@
         <f t="shared" ref="G5:G33" si="5">((F5-F4)*TEMP_RATE+MESCLUN_FERT)</f>
         <v>1690.791015625</v>
       </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I5">
+        <f t="shared" ref="I5:I23" si="6">(MIN(B5,OWNER_HRS)*OWNER_RATE+MAX(0,B5-OWNER_HRS)*TEMP_RATE)-(MIN(B4,OWNER_HRS)*OWNER_RATE+MAX(0,B4-OWNER_HRS)*TEMP_RATE)+TOMATO_FERT</f>
+        <v>5005</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>3</v>
       </c>
@@ -1840,8 +1864,12 @@
         <f t="shared" si="5"/>
         <v>1710.9371948242183</v>
       </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I6">
+        <f t="shared" si="6"/>
+        <v>5795.6250000000027</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>4</v>
       </c>
@@ -1869,8 +1897,12 @@
         <f t="shared" si="5"/>
         <v>1731.460342407227</v>
       </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I7">
+        <f t="shared" si="6"/>
+        <v>6703.125</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>5</v>
       </c>
@@ -1898,8 +1930,12 @@
         <f t="shared" si="5"/>
         <v>1752.3667347431174</v>
       </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I8">
+        <f t="shared" si="6"/>
+        <v>7660.859375</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>6</v>
       </c>
@@ -1927,8 +1963,12 @@
         <f t="shared" si="5"/>
         <v>1773.6627462089068</v>
       </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I9">
+        <f t="shared" si="6"/>
+        <v>4906.2750000000051</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>7</v>
       </c>
@@ -1956,8 +1996,12 @@
         <f t="shared" si="5"/>
         <v>1795.3548506590337</v>
       </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I10">
+        <f t="shared" si="6"/>
+        <v>5585.7089062500017</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>8</v>
       </c>
@@ -1985,8 +2029,12 @@
         <f t="shared" si="5"/>
         <v>1817.4496229163231</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I11">
+        <f t="shared" si="6"/>
+        <v>6360.7668437500033</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>9</v>
       </c>
@@ -2014,8 +2062,12 @@
         <f t="shared" si="5"/>
         <v>1839.9537402846258</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I12">
+        <f t="shared" si="6"/>
+        <v>7243.7792796875074</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>10</v>
       </c>
@@ -2043,8 +2095,12 @@
         <f t="shared" si="5"/>
         <v>1862.8739840835569</v>
       </c>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I13">
+        <f t="shared" si="6"/>
+        <v>8248.586534375012</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>11</v>
       </c>
@@ -2072,8 +2128,12 @@
         <f t="shared" si="5"/>
         <v>1886.2172412055384</v>
       </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I14">
+        <f t="shared" si="6"/>
+        <v>9390.7174472031329</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>12</v>
       </c>
@@ -2101,8 +2161,12 @@
         <f t="shared" si="5"/>
         <v>1909.9905056955636</v>
       </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I15">
+        <f t="shared" si="6"/>
+        <v>10687.58867725313</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>13</v>
       </c>
@@ -2130,8 +2194,12 @@
         <f t="shared" si="5"/>
         <v>1934.2008803538927</v>
       </c>
-    </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I16">
+        <f t="shared" si="6"/>
+        <v>12158.726978841107</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A17">
         <v>14</v>
       </c>
@@ -2159,8 +2227,12 @@
         <f t="shared" si="5"/>
         <v>1958.8555783621748</v>
       </c>
-    </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I17">
+        <f t="shared" si="6"/>
+        <v>13826.017053974152</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A18">
         <v>15</v>
       </c>
@@ -2188,8 +2260,12 @@
         <f t="shared" si="5"/>
         <v>1983.961924933097</v>
       </c>
-    </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I18">
+        <f t="shared" si="6"/>
+        <v>15713.977874345364</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A19">
         <v>16</v>
       </c>
@@ -2217,8 +2293,12 @@
         <f t="shared" si="5"/>
         <v>2009.527358984185</v>
       </c>
-    </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I19">
+        <f t="shared" si="6"/>
+        <v>17850.0706882511</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A20">
         <v>17</v>
       </c>
@@ -2246,8 +2326,12 @@
         <f t="shared" si="5"/>
         <v>2035.5594348357702</v>
       </c>
-    </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I20">
+        <f t="shared" si="6"/>
+        <v>20265.042286194526</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A21">
         <v>18</v>
       </c>
@@ -2275,8 +2359,12 @@
         <f t="shared" si="5"/>
         <v>2062.0658239338081</v>
       </c>
-    </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I21">
+        <f t="shared" si="6"/>
+        <v>22993.307496844121</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A22">
         <v>19</v>
       </c>
@@ -2304,8 +2392,12 @@
         <f t="shared" si="5"/>
         <v>2089.0543165975987</v>
       </c>
-    </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I22">
+        <f t="shared" si="6"/>
+        <v>26073.375326761772</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A23">
         <v>20</v>
       </c>
@@ -2333,8 +2425,12 @@
         <f t="shared" si="5"/>
         <v>2116.5328237930053</v>
       </c>
-    </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="I23">
+        <f t="shared" si="6"/>
+        <v>29548.323647694342</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A24">
         <v>21</v>
       </c>
@@ -2347,7 +2443,7 @@
         <v>2144.5093789313141</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A25">
         <v>22</v>
       </c>
@@ -2360,7 +2456,7 @@
         <v>2172.9921396943791</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A26">
         <v>23</v>
       </c>
@@ -2373,7 +2469,7 @@
         <v>2201.9893898860491</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A27">
         <v>24</v>
       </c>
@@ -2386,7 +2482,7 @@
         <v>2231.5095413106928</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A28">
         <v>25</v>
       </c>
@@ -2399,7 +2495,7 @@
         <v>2261.5611356787767</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A29">
         <v>26</v>
       </c>
@@ -2412,7 +2508,7 @@
         <v>2292.1528465402416</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A30">
         <v>27</v>
       </c>
@@ -2425,7 +2521,7 @@
         <v>2323.2934812457729</v>
       </c>
     </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A31">
         <v>28</v>
       </c>
@@ -2438,7 +2534,7 @@
         <v>2354.9919829366972</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A32">
         <v>29</v>
       </c>
@@ -2466,13 +2562,28 @@
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B35" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C35" t="s">
-        <v>101</v>
+        <v>102</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A39" t="s">
+        <v>105</v>
       </c>
     </row>
   </sheetData>
@@ -2493,21 +2604,21 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B2">
         <v>99</v>
@@ -2523,10 +2634,10 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="B3" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="C3">
         <f>TOMATO_BEDS+CARROT_BEDS+MESCLUN_BEDS</f>
@@ -2539,10 +2650,10 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="B4" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C4">
         <f>TOMATO_BEDS</f>
@@ -2555,10 +2666,10 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="B5" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C5">
         <f>CARROT_BEDS</f>
@@ -2571,10 +2682,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="B6" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="C6">
         <f>MESCLUN_BEDS</f>
@@ -2587,10 +2698,10 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="B7" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="C7">
         <f>CostStructure!B14</f>
@@ -2603,18 +2714,18 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B8" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="C8" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="B9">
         <v>42762</v>
@@ -2630,26 +2741,26 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B11" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="B12" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="B13" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>